<commit_message>
Update berita 2026-08-05 05:34 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-07-29.xlsx
+++ b/data/berita_2026-07-29.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$H$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -430,6 +430,7 @@
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -473,6 +474,11 @@
           <t>Media</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Sentimen</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -511,6 +517,7 @@
           <t>Antara</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -549,9 +556,10 @@
           <t>Antara</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H3"/>
+  <autoFilter ref="A1:I3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>